<commit_message>
Implement static file serving and enhance token validation. Added multer for file uploads, updated token validation to use Authorization header, and improved player data routes to handle image uploads. Also, added a new route to verify token validity.
</commit_message>
<xml_diff>
--- a/storage/player_data.xlsx
+++ b/storage/player_data.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N28"/>
+  <dimension ref="A1:N34"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -454,7 +454,7 @@
         <v>Adam A.</v>
       </c>
       <c r="D2" t="str">
-        <v>null</v>
+        <v>Adam Aiman Shah</v>
       </c>
       <c r="E2" t="str">
         <v>RB</v>
@@ -476,6 +476,9 @@
       </c>
       <c r="K2">
         <v>0</v>
+      </c>
+      <c r="L2" t="str">
+        <v>2025-05-31T13:19:26.960Z</v>
       </c>
     </row>
     <row r="3">
@@ -629,7 +632,7 @@
         <v>Azam F.</v>
       </c>
       <c r="D7" t="str">
-        <v>null</v>
+        <v>Azam Fazly</v>
       </c>
       <c r="E7" t="str">
         <v>RW</v>
@@ -640,8 +643,8 @@
       <c r="G7">
         <v>24</v>
       </c>
-      <c r="H7">
-        <v>0</v>
+      <c r="H7" t="str">
+        <v>1</v>
       </c>
       <c r="I7">
         <v>0</v>
@@ -651,6 +654,9 @@
       </c>
       <c r="K7">
         <v>0</v>
+      </c>
+      <c r="L7" t="str">
+        <v>2025-05-31T13:20:16.542Z</v>
       </c>
     </row>
     <row r="8">
@@ -1394,15 +1400,210 @@
         <v>0</v>
       </c>
       <c r="L28" t="str">
-        <v>2025-05-25T09:24:16.319Z</v>
+        <v>2025-05-25T13:12:28.977Z</v>
+      </c>
+      <c r="M28" t="str">
+        <v>2025-05-25T13:12:28.977Z</v>
       </c>
       <c r="N28" t="str">
         <v>2025-05-25T09:22:30.917Z</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="L29" t="str">
+        <v>2025-05-25T13:08:33.100Z</v>
+      </c>
+      <c r="M29" t="str">
+        <v>2025-05-25T13:08:33.100Z</v>
+      </c>
+      <c r="N29" t="str">
+        <v>2025-05-25T12:24:39.060Z</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Neh</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Nazrin Amirrullah bin Zaidi</v>
+      </c>
+      <c r="E30" t="str">
+        <v>RB</v>
+      </c>
+      <c r="F30" t="str">
+        <v>R</v>
+      </c>
+      <c r="G30" t="str">
+        <v>24</v>
+      </c>
+      <c r="H30" t="str">
+        <v>1</v>
+      </c>
+      <c r="I30" t="str">
+        <v>0</v>
+      </c>
+      <c r="J30" t="str">
+        <v>0</v>
+      </c>
+      <c r="K30" t="str">
+        <v>0</v>
+      </c>
+      <c r="L30" t="str">
+        <v>2025-05-25T13:08:28.482Z</v>
+      </c>
+      <c r="M30" t="str">
+        <v>2025-05-25T13:08:28.482Z</v>
+      </c>
+      <c r="N30" t="str">
+        <v>2025-05-25T12:25:54.254Z</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="L31" t="str">
+        <v>2025-05-25T13:08:23.836Z</v>
+      </c>
+      <c r="M31" t="str">
+        <v>2025-05-25T13:08:23.836Z</v>
+      </c>
+      <c r="N31" t="str">
+        <v>2025-05-25T12:29:05.045Z</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="C32" t="str">
+        <v xml:space="preserve">Ali </v>
+      </c>
+      <c r="D32" t="str">
+        <v>Alialba</v>
+      </c>
+      <c r="E32" t="str">
+        <v>RB</v>
+      </c>
+      <c r="F32" t="str">
+        <v>L</v>
+      </c>
+      <c r="G32" t="str">
+        <v>23</v>
+      </c>
+      <c r="H32" t="str">
+        <v>13</v>
+      </c>
+      <c r="I32" t="str">
+        <v>2</v>
+      </c>
+      <c r="J32" t="str">
+        <v>44</v>
+      </c>
+      <c r="K32" t="str">
+        <v>123</v>
+      </c>
+      <c r="L32" t="str">
+        <v>2025-05-25T13:03:29.901Z</v>
+      </c>
+      <c r="M32" t="str">
+        <v>2025-05-25T13:03:29.901Z</v>
+      </c>
+      <c r="N32" t="str">
+        <v>2025-05-25T12:45:33.970Z</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="C33" t="str">
+        <v xml:space="preserve">Nazrin </v>
+      </c>
+      <c r="D33" t="str">
+        <v>Nazrin Amirrullah bin Zaidi</v>
+      </c>
+      <c r="E33" t="str">
+        <v>LB</v>
+      </c>
+      <c r="F33" t="str">
+        <v>R</v>
+      </c>
+      <c r="G33" t="str">
+        <v>24</v>
+      </c>
+      <c r="H33" t="str">
+        <v>1</v>
+      </c>
+      <c r="I33" t="str">
+        <v>2</v>
+      </c>
+      <c r="J33" t="str">
+        <v>3</v>
+      </c>
+      <c r="K33" t="str">
+        <v>5</v>
+      </c>
+      <c r="L33" t="str">
+        <v>2025-05-31T13:06:34.459Z</v>
+      </c>
+      <c r="M33" t="str">
+        <v>2025-05-31T13:06:34.459Z</v>
+      </c>
+      <c r="N33" t="str">
+        <v>2025-05-31T12:52:48.862Z</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="C34" t="str">
+        <v>asdasdasd</v>
+      </c>
+      <c r="D34" t="str">
+        <v>asdasdasd</v>
+      </c>
+      <c r="E34" t="str">
+        <v>CB</v>
+      </c>
+      <c r="F34" t="str">
+        <v>R</v>
+      </c>
+      <c r="G34" t="str">
+        <v>23</v>
+      </c>
+      <c r="H34" t="str">
+        <v>1</v>
+      </c>
+      <c r="I34" t="str">
+        <v>3</v>
+      </c>
+      <c r="J34" t="str">
+        <v>4</v>
+      </c>
+      <c r="K34" t="str">
+        <v>5</v>
+      </c>
+      <c r="L34" t="str">
+        <v>2025-05-31T13:06:31.551Z</v>
+      </c>
+      <c r="M34" t="str">
+        <v>2025-05-31T13:06:31.551Z</v>
+      </c>
+      <c r="N34" t="str">
+        <v>2025-05-31T12:58:45.381Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N34"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>